<commit_message>
Move dependencies to right place
</commit_message>
<xml_diff>
--- a/master_workbook.xlsx
+++ b/master_workbook.xlsx
@@ -520,7 +520,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F78"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -2090,7 +2090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2113,6 +2113,114 @@
         <is>
           <t>IsActive</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>500</v>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sanduiche</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Trento</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>400</v>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Coca lata</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>600</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2126,7 +2234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2144,6 +2252,81 @@
         <is>
           <t>IsActive</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bruno</t>
+        </is>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="C4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Davi</t>
+        </is>
+      </c>
+      <c r="C5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>S005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Eduardo</t>
+        </is>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2157,7 +2340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2217,6 +2400,1901 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>20260808020518523423</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:18.523423+00:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>RESTOCK</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-20000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>20260808020518901880</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:18.901880+00:00</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>RESTOCK</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>80</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-40000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>20260808020519282677</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:19.282677+00:00</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>RESTOCK</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-35000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>20260808020519659173</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:19.659173+00:00</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>RESTOCK</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>120</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-24000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>20260808020520041294</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:20.041294+00:00</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>RESTOCK</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>S005</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>90</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-27000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>20260808020520426191</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:20.426191+00:00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>RESTOCK</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>50</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-10000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>20260808020520813190</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:20.813190+00:00</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>20260808020521197317</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:21.197317+00:00</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>20260808020521585418</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:21.585418+00:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>20260808020521965178</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:21.965178+00:00</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>-5</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>20260808020522350119</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:22.350119+00:00</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>S005</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>-4</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>20260808020522729164</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:22.729164+00:00</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>-3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1800</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>20260808020523111935</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:23.111935+00:00</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>20260808020523495232</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:23.495232+00:00</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>20260808020523879975</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:23.879975+00:00</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>OnCredit</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>-10</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Tab para dep. A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>20260808020524605476</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:24.605476+00:00</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>S005</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>OnCredit</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>-4</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Tab para un. B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>20260808020525340117</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:25.340117+00:00</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>OnCredit</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>-5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Monster fiado para Vanessa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>20260808020526050089</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:26.050089+00:00</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>OnCredit</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>-6</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Turma de BCC com pressa</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>20260808020526760386</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:26.760386+00:00</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>-10</v>
+      </c>
+      <c r="H20" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Pagamento com o vaucher brinde</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20260808020527151399</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:27.151399+00:00</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>-3</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Desconto de funcionário</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>20260808020527541636</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:27.541636+00:00</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>S005</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>-4</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Desconto de functionário</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>20260808020527936222</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:27.936222+00:00</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CREDIT_PAYMENT</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>2500</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>20260808020523879975</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Pagamento parcial dep. A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>20260808020528324504</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:28.324504+00:00</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CREDIT_PAYMENT</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>20260808020524605476</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Pagamento parcial un. B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>20260808020528715783</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:28.715783+00:00</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CREDIT_PAYMENT</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>20260808020525340117</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>20260808020529102707</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:29.102707+00:00</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CREDIT_PAYMENT</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>3600</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>20260808020526050089</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>20260808020529498383</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:29.498383+00:00</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>WRITE_OFF</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Sanduíche vencido</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>20260808020529896619</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:29.896619+00:00</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>WRITE_OFF</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Derramou o café</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>20260808020530296392</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:30.296392+00:00</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>WRITE_OFF</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>-3</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Pacote rasgado</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>20260808020530690111</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:30.690111+00:00</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H30" t="n">
+        <v>500</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>20260808020531423016</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:31.423016+00:00</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>VOID</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="n">
+        <v>-500</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>20260808020530690111</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Vendi errado</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>20260808020531831686</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:31.831686+00:00</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>RESTOCK</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>10</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-3000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>20260808020532552005</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:32.552005+00:00</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>VOID</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>-10</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>20260808020531831686</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Reestoque duplicado</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>20260808020532945406</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:32.945406+00:00</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H34" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>20260808020533673870</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:05:33.673870+00:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>VOID</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>20260808020532945406</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Não era no PIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>20260808020729294597</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:07:29.294597+00:00</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>RESTOCK</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>100</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>-10000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>20260808021251246705</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:12:51.246705+00:00</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>20260808021706395005</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:17:06.395005+00:00</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H38" t="n">
+        <v>2</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>20260808022102951189</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:21:02.951189+00:00</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>20260808023447247957</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:34:47.247957+00:00</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H40" t="n">
+        <v>2</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>20260808023710762458</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:37:10.762458+00:00</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>20260808024246469881</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:42:46.469881+00:00</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>20260808024503152560</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:45:03.152560+00:00</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H43" t="n">
+        <v>2</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>20260808025600017782</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-08-08T02:56:00.017782+00:00</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H44" t="n">
+        <v>2</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>20260808030317274165</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-08-08T03:03:17.274165+00:00</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>20260808030317274460</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-08-08T03:03:17.274460+00:00</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H46" t="n">
+        <v>600</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>